<commit_message>
decreased the console output, ready for multiprocessing now
</commit_message>
<xml_diff>
--- a/processed_data/nikon_cellpose_bags_spots_results.xlsx
+++ b/processed_data/nikon_cellpose_bags_spots_results.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,56 +426,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ROI</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Spot_Count</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ROI_Area_pixels</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ROI_Area_um2</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>ROI_Volume_um3</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Spots_per_Area</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Spots_per_Volume</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Experiment</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Image_Number</t>
         </is>
@@ -477,19 +489,19 @@
         <v>439</v>
       </c>
       <c r="C2" t="n">
-        <v>269320</v>
+        <v>269420</v>
       </c>
       <c r="D2" t="n">
-        <v>14031.62189164888</v>
+        <v>14036.83191017393</v>
       </c>
       <c r="E2" t="n">
-        <v>280632.4378329777</v>
+        <v>280736.6382034785</v>
       </c>
       <c r="F2" t="n">
-        <v>0.03128647588923965</v>
+        <v>0.0312748633601441</v>
       </c>
       <c r="G2" t="n">
-        <v>0.001564323794461982</v>
+        <v>0.001563743168007205</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -585,19 +597,19 @@
         <v>723</v>
       </c>
       <c r="C5" t="n">
-        <v>478100</v>
+        <v>478200</v>
       </c>
       <c r="D5" t="n">
-        <v>24909.09856823604</v>
+        <v>24914.30858676109</v>
       </c>
       <c r="E5" t="n">
-        <v>498181.9713647208</v>
+        <v>498286.1717352218</v>
       </c>
       <c r="F5" t="n">
-        <v>0.02902553852036886</v>
+        <v>0.0290194687716193</v>
       </c>
       <c r="G5" t="n">
-        <v>0.001451276926018443</v>
+        <v>0.001450973438580965</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -621,19 +633,19 @@
         <v>697</v>
       </c>
       <c r="C6" t="n">
-        <v>480630</v>
+        <v>480230</v>
       </c>
       <c r="D6" t="n">
-        <v>25040.91203691966</v>
+        <v>25020.07196281948</v>
       </c>
       <c r="E6" t="n">
-        <v>500818.2407383932</v>
+        <v>500401.4392563896</v>
       </c>
       <c r="F6" t="n">
-        <v>0.02783444943907641</v>
+        <v>0.0278576337044818</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00139172247195382</v>
+        <v>0.00139288168522409</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -657,19 +669,19 @@
         <v>680</v>
       </c>
       <c r="C7" t="n">
-        <v>418230</v>
+        <v>418140</v>
       </c>
       <c r="D7" t="n">
-        <v>21789.86047729211</v>
+        <v>21785.17146061957</v>
       </c>
       <c r="E7" t="n">
-        <v>435797.2095458423</v>
+        <v>435703.4292123915</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03120717549837683</v>
+        <v>0.03121389249697742</v>
       </c>
       <c r="G7" t="n">
-        <v>0.001560358774918841</v>
+        <v>0.001560694624848871</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -693,19 +705,19 @@
         <v>801</v>
       </c>
       <c r="C8" t="n">
-        <v>604300</v>
+        <v>604100</v>
       </c>
       <c r="D8" t="n">
-        <v>31484.14194684175</v>
+        <v>31473.72190979166</v>
       </c>
       <c r="E8" t="n">
-        <v>629682.8389368349</v>
+        <v>629474.4381958332</v>
       </c>
       <c r="F8" t="n">
-        <v>0.02544137938878624</v>
+        <v>0.02544980229207669</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001272068969439312</v>
+        <v>0.001272490114603834</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -729,19 +741,19 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>535894</v>
+        <v>535994</v>
       </c>
       <c r="D9" t="n">
-        <v>27920.17667460005</v>
+        <v>27925.3866931251</v>
       </c>
       <c r="E9" t="n">
-        <v>558403.5334920011</v>
+        <v>558507.7338625019</v>
       </c>
       <c r="F9" t="n">
-        <v>0.004297967072291778</v>
+        <v>0.004297165203787226</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0002148983536145889</v>
+        <v>0.0002148582601893613</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -795,61 +807,61 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" t="n">
+        <v>97</v>
+      </c>
+      <c r="C11" t="n">
+        <v>520345</v>
+      </c>
+      <c r="D11" t="n">
+        <v>27110.07089414094</v>
+      </c>
+      <c r="E11" t="n">
+        <v>542201.4178828187</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.003578006135755394</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0001789003067877697</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nikon_cellpose_bags_spots</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>P_None_No</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
         <v>2</v>
-      </c>
-      <c r="B11" t="n">
-        <v>114</v>
-      </c>
-      <c r="C11" t="n">
-        <v>565643</v>
-      </c>
-      <c r="D11" t="n">
-        <v>29470.10508561544</v>
-      </c>
-      <c r="E11" t="n">
-        <v>589402.1017123087</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.003868326891567285</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.0001934163445783643</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nikon_cellpose_bags_spots</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>P_None_No</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B12" t="n">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="C12" t="n">
-        <v>267342</v>
+        <v>565443</v>
       </c>
       <c r="D12" t="n">
-        <v>13928.56772522351</v>
+        <v>29459.68504856534</v>
       </c>
       <c r="E12" t="n">
-        <v>278571.3545044702</v>
+        <v>589193.7009713069</v>
       </c>
       <c r="F12" t="n">
-        <v>0.006533335070425537</v>
+        <v>0.003869695138018853</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0003266667535212769</v>
+        <v>0.0001934847569009426</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -862,30 +874,30 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B13" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="C13" t="n">
-        <v>281652</v>
+        <v>265642</v>
       </c>
       <c r="D13" t="n">
-        <v>14674.12137615733</v>
+        <v>13839.99741029776</v>
       </c>
       <c r="E13" t="n">
-        <v>293482.4275231465</v>
+        <v>276799.9482059552</v>
       </c>
       <c r="F13" t="n">
-        <v>0.007359895507984525</v>
+        <v>0.006502891390213324</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0003679947753992263</v>
+        <v>0.0003251445695106662</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -903,25 +915,25 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B14" t="n">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="C14" t="n">
-        <v>269392</v>
+        <v>281452</v>
       </c>
       <c r="D14" t="n">
-        <v>14035.37310498691</v>
+        <v>14663.70133910724</v>
       </c>
       <c r="E14" t="n">
-        <v>280707.4620997383</v>
+        <v>293274.0267821447</v>
       </c>
       <c r="F14" t="n">
-        <v>0.008692323252643146</v>
+        <v>0.007365125455192563</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0004346161626321573</v>
+        <v>0.0003682562727596282</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -942,22 +954,22 @@
         <v>3</v>
       </c>
       <c r="B15" t="n">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C15" t="n">
-        <v>416163</v>
+        <v>269592</v>
       </c>
       <c r="D15" t="n">
-        <v>21682.16939437945</v>
+        <v>14045.793142037</v>
       </c>
       <c r="E15" t="n">
-        <v>433643.3878875891</v>
+        <v>280915.8628407401</v>
       </c>
       <c r="F15" t="n">
-        <v>0.005257776467217879</v>
+        <v>0.008685874750274648</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0002628888233608939</v>
+        <v>0.0004342937375137323</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -970,7 +982,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -978,22 +990,22 @@
         <v>3</v>
       </c>
       <c r="B16" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C16" t="n">
-        <v>481085</v>
+        <v>416063</v>
       </c>
       <c r="D16" t="n">
-        <v>25064.61762120861</v>
+        <v>21676.95937585441</v>
       </c>
       <c r="E16" t="n">
-        <v>501292.3524241722</v>
+        <v>433539.1875170881</v>
       </c>
       <c r="F16" t="n">
-        <v>0.004588141009687373</v>
+        <v>0.005259040164414509</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0002294070504843687</v>
+        <v>0.0002629520082207255</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1006,30 +1018,30 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B17" t="n">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C17" t="n">
-        <v>454033</v>
+        <v>481085</v>
       </c>
       <c r="D17" t="n">
-        <v>23655.20340981367</v>
+        <v>25064.61762120861</v>
       </c>
       <c r="E17" t="n">
-        <v>473104.0681962734</v>
+        <v>501292.3524241722</v>
       </c>
       <c r="F17" t="n">
-        <v>0.005199701641498963</v>
+        <v>0.004588141009687373</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0002599850820749481</v>
+        <v>0.0002294070504843687</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1047,25 +1059,25 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" t="n">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="C18" t="n">
-        <v>439263</v>
+        <v>454333</v>
       </c>
       <c r="D18" t="n">
-        <v>22885.68367366465</v>
+        <v>23670.8334653888</v>
       </c>
       <c r="E18" t="n">
-        <v>457713.673473293</v>
+        <v>473416.669307776</v>
       </c>
       <c r="F18" t="n">
-        <v>0.005680407098766095</v>
+        <v>0.005196268233640741</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0002840203549383048</v>
+        <v>0.0002598134116820371</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1083,25 +1095,25 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B19" t="n">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C19" t="n">
-        <v>750346</v>
+        <v>439463</v>
       </c>
       <c r="D19" t="n">
-        <v>39093.16560192771</v>
+        <v>22896.10371071474</v>
       </c>
       <c r="E19" t="n">
-        <v>781863.3120385543</v>
+        <v>457922.0742142948</v>
       </c>
       <c r="F19" t="n">
-        <v>0.003120750088194037</v>
+        <v>0.005677821940471191</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0001560375044097018</v>
+        <v>0.0002838910970235596</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1114,30 +1126,30 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" t="n">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C20" t="n">
-        <v>717257</v>
+        <v>750346</v>
       </c>
       <c r="D20" t="n">
-        <v>37369.22257217586</v>
+        <v>39093.16560192771</v>
       </c>
       <c r="E20" t="n">
-        <v>747384.4514435171</v>
+        <v>781863.3120385543</v>
       </c>
       <c r="F20" t="n">
-        <v>0.003505558611688624</v>
+        <v>0.003120750088194037</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0001752779305844312</v>
+        <v>0.0001560375044097018</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1155,25 +1167,25 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B21" t="n">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="C21" t="n">
-        <v>375962</v>
+        <v>717057</v>
       </c>
       <c r="D21" t="n">
-        <v>19587.68984712646</v>
+        <v>37358.80253512577</v>
       </c>
       <c r="E21" t="n">
-        <v>391753.7969425292</v>
+        <v>747176.0507025155</v>
       </c>
       <c r="F21" t="n">
-        <v>0.006177349189432407</v>
+        <v>0.003506536374575448</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0003088674594716203</v>
+        <v>0.0001753268187287724</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1186,30 +1198,30 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="C22" t="n">
-        <v>348514</v>
+        <v>375962</v>
       </c>
       <c r="D22" t="n">
-        <v>18157.64396237234</v>
+        <v>19587.68984712646</v>
       </c>
       <c r="E22" t="n">
-        <v>363152.8792474468</v>
+        <v>391753.7969425292</v>
       </c>
       <c r="F22" t="n">
-        <v>0.005892835007764971</v>
+        <v>0.006177349189432407</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0002946417503882486</v>
+        <v>0.0003088674594716203</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1227,25 +1239,25 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B23" t="n">
-        <v>7</v>
+        <v>107</v>
       </c>
       <c r="C23" t="n">
-        <v>286682</v>
+        <v>348514</v>
       </c>
       <c r="D23" t="n">
-        <v>14936.18530796705</v>
+        <v>18157.64396237234</v>
       </c>
       <c r="E23" t="n">
-        <v>298723.7061593409</v>
+        <v>363152.8792474468</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0004686604950104736</v>
+        <v>0.005892835007764971</v>
       </c>
       <c r="G23" t="n">
-        <v>2.343302475052368e-05</v>
+        <v>0.0002946417503882486</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1254,11 +1266,11 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>None_0</t>
+          <t>P_None_No</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -1266,34 +1278,106 @@
         <v>1</v>
       </c>
       <c r="B24" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" t="n">
+        <v>286682</v>
+      </c>
+      <c r="D24" t="n">
+        <v>14936.18530796705</v>
+      </c>
+      <c r="E24" t="n">
+        <v>298723.7061593409</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.0004686604950104736</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2.343302475052368e-05</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nikon_cellpose_bags_spots</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>None_0</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>461406</v>
+      </c>
+      <c r="D25" t="n">
+        <v>24039.33807566517</v>
+      </c>
+      <c r="E25" t="n">
+        <v>480786.7615133034</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4.159848315508704e-05</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2.079924157754351e-06</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nikon_cellpose_bags_spots</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>None_0</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" t="n">
         <v>6</v>
       </c>
-      <c r="C24" t="n">
-        <v>944338</v>
-      </c>
-      <c r="D24" t="n">
-        <v>49200.18473903135</v>
-      </c>
-      <c r="E24" t="n">
-        <v>984003.694780627</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.0001219507616043583</v>
-      </c>
-      <c r="G24" t="n">
-        <v>6.097538080217915e-06</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nikon_cellpose_bags_spots</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="C26" t="n">
+        <v>944638</v>
+      </c>
+      <c r="D26" t="n">
+        <v>49215.81479460648</v>
+      </c>
+      <c r="E26" t="n">
+        <v>984316.2958921295</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.0001219120322408547</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6.095601612042736e-06</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nikon_cellpose_bags_spots</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
         <is>
           <t>None_0</t>
         </is>
       </c>
-      <c r="J24" t="n">
+      <c r="J26" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1312,57 +1396,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Spot_Count_count</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Spot_Count_mean</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Spot_Count_std</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Spot_Count_sum</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ROI_Area_um2_mean</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ROI_Area_um2_std</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Spots_per_Area_mean</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Spots_per_Area_std</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Spots_per_Volume_mean</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Spots_per_Volume_std</t>
         </is>
@@ -1375,22 +1459,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>6.5</v>
+        <v>4.667</v>
       </c>
       <c r="D2" t="n">
-        <v>0.707</v>
+        <v>3.215</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" t="n">
-        <v>32068.185</v>
+        <v>29397.113</v>
       </c>
       <c r="G2" t="n">
-        <v>24228.306</v>
+        <v>17756.761</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1412,22 +1496,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>115.643</v>
+        <v>114.333</v>
       </c>
       <c r="D3" t="n">
-        <v>11.043</v>
+        <v>11.824</v>
       </c>
       <c r="E3" t="n">
-        <v>1619</v>
+        <v>1715</v>
       </c>
       <c r="F3" t="n">
-        <v>23763.378</v>
+        <v>23980.934</v>
       </c>
       <c r="G3" t="n">
-        <v>7852.325</v>
+        <v>7622.504</v>
       </c>
       <c r="H3" t="n">
         <v>0.005</v>
@@ -1461,10 +1545,10 @@
         <v>4553</v>
       </c>
       <c r="F4" t="n">
-        <v>22036.741</v>
+        <v>22033.094</v>
       </c>
       <c r="G4" t="n">
-        <v>5712.431</v>
+        <v>5706.991</v>
       </c>
       <c r="H4" t="n">
         <v>0.03</v>

</xml_diff>

<commit_message>
getting ready for cluster compatibility
</commit_message>
<xml_diff>
--- a/processed_data/nikon_cellpose_bags_spots_results.xlsx
+++ b/processed_data/nikon_cellpose_bags_spots_results.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,56 +414,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ROI</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Spot_Count</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ROI_Area_pixels</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ROI_Area_um2</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>ROI_Volume_um3</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Spots_per_Area</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Spots_per_Volume</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Experiment</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Image_Number</t>
         </is>
@@ -522,22 +510,22 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="C3" t="n">
-        <v>359670</v>
+        <v>359460</v>
       </c>
       <c r="D3" t="n">
-        <v>18738.87362902626</v>
+        <v>18727.93259012367</v>
       </c>
       <c r="E3" t="n">
-        <v>374777.4725805253</v>
+        <v>374558.6518024735</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03292620528932301</v>
+        <v>0.03299883727293568</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00164631026446615</v>
+        <v>0.001649941863646784</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -561,19 +549,19 @@
         <v>596</v>
       </c>
       <c r="C4" t="n">
-        <v>350530</v>
+        <v>350730</v>
       </c>
       <c r="D4" t="n">
-        <v>18262.67793583723</v>
+        <v>18273.09797288732</v>
       </c>
       <c r="E4" t="n">
-        <v>365253.5587167446</v>
+        <v>365461.9594577464</v>
       </c>
       <c r="F4" t="n">
-        <v>0.03263486341345685</v>
+        <v>0.03261625373455088</v>
       </c>
       <c r="G4" t="n">
-        <v>0.001631743170672842</v>
+        <v>0.001630812686727544</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -597,19 +585,19 @@
         <v>723</v>
       </c>
       <c r="C5" t="n">
-        <v>478200</v>
+        <v>478600</v>
       </c>
       <c r="D5" t="n">
-        <v>24914.30858676109</v>
+        <v>24935.14866086126</v>
       </c>
       <c r="E5" t="n">
-        <v>498286.1717352218</v>
+        <v>498702.9732172252</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0290194687716193</v>
+        <v>0.02899521514122096</v>
       </c>
       <c r="G5" t="n">
-        <v>0.001450973438580965</v>
+        <v>0.001449760757061048</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -630,22 +618,22 @@
         <v>1</v>
       </c>
       <c r="B6" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C6" t="n">
-        <v>480230</v>
+        <v>480730</v>
       </c>
       <c r="D6" t="n">
-        <v>25020.07196281948</v>
+        <v>25046.1220554447</v>
       </c>
       <c r="E6" t="n">
-        <v>500401.4392563896</v>
+        <v>500922.4411088941</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0278576337044818</v>
+        <v>0.02786858574173018</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00139288168522409</v>
+        <v>0.001393429287086509</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -669,19 +657,19 @@
         <v>680</v>
       </c>
       <c r="C7" t="n">
-        <v>418140</v>
+        <v>418230</v>
       </c>
       <c r="D7" t="n">
-        <v>21785.17146061957</v>
+        <v>21789.86047729211</v>
       </c>
       <c r="E7" t="n">
-        <v>435703.4292123915</v>
+        <v>435797.2095458423</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03121389249697742</v>
+        <v>0.03120717549837683</v>
       </c>
       <c r="G7" t="n">
-        <v>0.001560694624848871</v>
+        <v>0.001560358774918841</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -705,19 +693,19 @@
         <v>801</v>
       </c>
       <c r="C8" t="n">
-        <v>604100</v>
+        <v>604300</v>
       </c>
       <c r="D8" t="n">
-        <v>31473.72190979166</v>
+        <v>31484.14194684175</v>
       </c>
       <c r="E8" t="n">
-        <v>629474.4381958332</v>
+        <v>629682.8389368349</v>
       </c>
       <c r="F8" t="n">
-        <v>0.02544980229207669</v>
+        <v>0.02544137938878624</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001272490114603834</v>
+        <v>0.001272068969439312</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -741,19 +729,19 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>535994</v>
+        <v>535884</v>
       </c>
       <c r="D9" t="n">
-        <v>27925.3866931251</v>
+        <v>27919.65567274755</v>
       </c>
       <c r="E9" t="n">
-        <v>558507.7338625019</v>
+        <v>558393.113454951</v>
       </c>
       <c r="F9" t="n">
-        <v>0.004297165203787226</v>
+        <v>0.004298047275602053</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0002148582601893613</v>
+        <v>0.0002149023637801026</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -774,22 +762,22 @@
         <v>2</v>
       </c>
       <c r="B10" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C10" t="n">
-        <v>482984</v>
+        <v>482884</v>
       </c>
       <c r="D10" t="n">
-        <v>25163.5558729992</v>
+        <v>25158.34585447416</v>
       </c>
       <c r="E10" t="n">
-        <v>503271.1174599839</v>
+        <v>503166.9170894831</v>
       </c>
       <c r="F10" t="n">
-        <v>0.004013741162407584</v>
+        <v>0.004054320605575916</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0002006870581203792</v>
+        <v>0.0002027160302787958</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -813,19 +801,19 @@
         <v>97</v>
       </c>
       <c r="C11" t="n">
-        <v>520345</v>
+        <v>520545</v>
       </c>
       <c r="D11" t="n">
-        <v>27110.07089414094</v>
+        <v>27120.49093119103</v>
       </c>
       <c r="E11" t="n">
-        <v>542201.4178828187</v>
+        <v>542409.8186238206</v>
       </c>
       <c r="F11" t="n">
-        <v>0.003578006135755394</v>
+        <v>0.003576631420356819</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0001789003067877697</v>
+        <v>0.000178831571017841</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -885,19 +873,19 @@
         <v>90</v>
       </c>
       <c r="C13" t="n">
-        <v>265642</v>
+        <v>264842</v>
       </c>
       <c r="D13" t="n">
-        <v>13839.99741029776</v>
+        <v>13798.31726209741</v>
       </c>
       <c r="E13" t="n">
-        <v>276799.9482059552</v>
+        <v>275966.3452419481</v>
       </c>
       <c r="F13" t="n">
-        <v>0.006502891390213324</v>
+        <v>0.006522534472172268</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0003251445695106662</v>
+        <v>0.0003261267236086134</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -921,19 +909,19 @@
         <v>108</v>
       </c>
       <c r="C14" t="n">
-        <v>281452</v>
+        <v>281352</v>
       </c>
       <c r="D14" t="n">
-        <v>14663.70133910724</v>
+        <v>14658.49132058219</v>
       </c>
       <c r="E14" t="n">
-        <v>293274.0267821447</v>
+        <v>293169.8264116439</v>
       </c>
       <c r="F14" t="n">
-        <v>0.007365125455192563</v>
+        <v>0.00736774321709054</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0003682562727596282</v>
+        <v>0.0003683871608545269</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -957,19 +945,19 @@
         <v>122</v>
       </c>
       <c r="C15" t="n">
-        <v>269592</v>
+        <v>269392</v>
       </c>
       <c r="D15" t="n">
-        <v>14045.793142037</v>
+        <v>14035.37310498691</v>
       </c>
       <c r="E15" t="n">
-        <v>280915.8628407401</v>
+        <v>280707.4620997383</v>
       </c>
       <c r="F15" t="n">
-        <v>0.008685874750274648</v>
+        <v>0.008692323252643146</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0004342937375137323</v>
+        <v>0.0004346161626321573</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -993,19 +981,19 @@
         <v>114</v>
       </c>
       <c r="C16" t="n">
-        <v>416063</v>
+        <v>415863</v>
       </c>
       <c r="D16" t="n">
-        <v>21676.95937585441</v>
+        <v>21666.53933880432</v>
       </c>
       <c r="E16" t="n">
-        <v>433539.1875170881</v>
+        <v>433330.7867760864</v>
       </c>
       <c r="F16" t="n">
-        <v>0.005259040164414509</v>
+        <v>0.005261569382048401</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0002629520082207255</v>
+        <v>0.00026307846910242</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1065,19 +1053,19 @@
         <v>123</v>
       </c>
       <c r="C18" t="n">
-        <v>454333</v>
+        <v>454233</v>
       </c>
       <c r="D18" t="n">
-        <v>23670.8334653888</v>
+        <v>23665.62344686376</v>
       </c>
       <c r="E18" t="n">
-        <v>473416.669307776</v>
+        <v>473312.4689372751</v>
       </c>
       <c r="F18" t="n">
-        <v>0.005196268233640741</v>
+        <v>0.005197412199013939</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0002598134116820371</v>
+        <v>0.000259870609950697</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1101,19 +1089,19 @@
         <v>130</v>
       </c>
       <c r="C19" t="n">
-        <v>439463</v>
+        <v>439263</v>
       </c>
       <c r="D19" t="n">
-        <v>22896.10371071474</v>
+        <v>22885.68367366465</v>
       </c>
       <c r="E19" t="n">
-        <v>457922.0742142948</v>
+        <v>457713.673473293</v>
       </c>
       <c r="F19" t="n">
-        <v>0.005677821940471191</v>
+        <v>0.005680407098766095</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0002838910970235596</v>
+        <v>0.0002840203549383048</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1137,19 +1125,19 @@
         <v>122</v>
       </c>
       <c r="C20" t="n">
-        <v>750346</v>
+        <v>750146</v>
       </c>
       <c r="D20" t="n">
-        <v>39093.16560192771</v>
+        <v>39082.74556487763</v>
       </c>
       <c r="E20" t="n">
-        <v>781863.3120385543</v>
+        <v>781654.9112975526</v>
       </c>
       <c r="F20" t="n">
-        <v>0.003120750088194037</v>
+        <v>0.00312158212624748</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0001560375044097018</v>
+        <v>0.000156079106312374</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1173,19 +1161,19 @@
         <v>131</v>
       </c>
       <c r="C21" t="n">
-        <v>717057</v>
+        <v>717457</v>
       </c>
       <c r="D21" t="n">
-        <v>37358.80253512577</v>
+        <v>37379.64260922595</v>
       </c>
       <c r="E21" t="n">
-        <v>747176.0507025155</v>
+        <v>747592.8521845189</v>
       </c>
       <c r="F21" t="n">
-        <v>0.003506536374575448</v>
+        <v>0.003504581393928761</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0001753268187287724</v>
+        <v>0.0001752290696964381</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1206,22 +1194,22 @@
         <v>1</v>
       </c>
       <c r="B22" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C22" t="n">
-        <v>375962</v>
+        <v>375462</v>
       </c>
       <c r="D22" t="n">
-        <v>19587.68984712646</v>
+        <v>19561.63975450124</v>
       </c>
       <c r="E22" t="n">
-        <v>391753.7969425292</v>
+        <v>391232.7950900247</v>
       </c>
       <c r="F22" t="n">
-        <v>0.006177349189432407</v>
+        <v>0.006134455061334383</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0003088674594716203</v>
+        <v>0.0003067227530667192</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1245,19 +1233,19 @@
         <v>107</v>
       </c>
       <c r="C23" t="n">
-        <v>348514</v>
+        <v>348404</v>
       </c>
       <c r="D23" t="n">
-        <v>18157.64396237234</v>
+        <v>18151.91294199479</v>
       </c>
       <c r="E23" t="n">
-        <v>363152.8792474468</v>
+        <v>363038.2588398958</v>
       </c>
       <c r="F23" t="n">
-        <v>0.005892835007764971</v>
+        <v>0.005894695525585817</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0002946417503882486</v>
+        <v>0.0002947347762792909</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1314,22 +1302,22 @@
         <v>1</v>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C25" t="n">
-        <v>461406</v>
+        <v>947638</v>
       </c>
       <c r="D25" t="n">
-        <v>24039.33807566517</v>
+        <v>49372.1153503578</v>
       </c>
       <c r="E25" t="n">
-        <v>480786.7615133034</v>
+        <v>987442.3070071561</v>
       </c>
       <c r="F25" t="n">
-        <v>4.159848315508704e-05</v>
+        <v>0.0001215260872948705</v>
       </c>
       <c r="G25" t="n">
-        <v>2.079924157754351e-06</v>
+        <v>6.076304364743527e-06</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1342,42 +1330,6 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" t="n">
-        <v>6</v>
-      </c>
-      <c r="C26" t="n">
-        <v>944638</v>
-      </c>
-      <c r="D26" t="n">
-        <v>49215.81479460648</v>
-      </c>
-      <c r="E26" t="n">
-        <v>984316.2958921295</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0.0001219120322408547</v>
-      </c>
-      <c r="G26" t="n">
-        <v>6.095601612042736e-06</v>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nikon_cellpose_bags_spots</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>None_0</t>
-        </is>
-      </c>
-      <c r="J26" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1396,57 +1348,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Spot_Count_count</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Spot_Count_mean</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spot_Count_std</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Spot_Count_sum</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ROI_Area_um2_mean</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ROI_Area_um2_std</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Spots_per_Area_mean</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Spots_per_Area_std</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Spots_per_Volume_mean</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Spots_per_Volume_std</t>
         </is>
@@ -1459,22 +1411,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>4.667</v>
+        <v>6.5</v>
       </c>
       <c r="D2" t="n">
-        <v>3.215</v>
+        <v>0.707</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
-        <v>29397.113</v>
+        <v>32154.15</v>
       </c>
       <c r="G2" t="n">
-        <v>17756.761</v>
+        <v>24349.88</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1502,16 +1454,16 @@
         <v>114.333</v>
       </c>
       <c r="D3" t="n">
-        <v>11.824</v>
+        <v>11.709</v>
       </c>
       <c r="E3" t="n">
         <v>1715</v>
       </c>
       <c r="F3" t="n">
-        <v>23980.934</v>
+        <v>23973.918</v>
       </c>
       <c r="G3" t="n">
-        <v>7622.504</v>
+        <v>7630.802</v>
       </c>
       <c r="H3" t="n">
         <v>0.005</v>
@@ -1536,19 +1488,19 @@
         <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>650.429</v>
+        <v>650.7140000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>115.299</v>
+        <v>115.319</v>
       </c>
       <c r="E4" t="n">
-        <v>4553</v>
+        <v>4555</v>
       </c>
       <c r="F4" t="n">
-        <v>22033.094</v>
+        <v>22041.877</v>
       </c>
       <c r="G4" t="n">
-        <v>5706.991</v>
+        <v>5713.771</v>
       </c>
       <c r="H4" t="n">
         <v>0.03</v>

</xml_diff>